<commit_message>
Metrics blueprint (v1) + align input schema to it
- docs/metrics-blueprint.md: decided spec — rich-but-honest box-score metrics
  (TS%/eFG%, per-36, AST:TO, scoring mix, DMV cohort percentiles, trend),
  archetype tags + GP-gated trajectory (no composite rating), self-reported vs
  Prospera-Verified measurables, records/milestones, v1 player-page layout, and
  honesty guardrails.
- Input schema: minutes emphasized + optional started/dfl/chg extras in the coach
  workbook and importer (pass-through to game logs; season GS when tracked).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Hayfield-Stats-Intake.xlsx
+++ b/docs/Hayfield-Stats-Intake.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -174,6 +174,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -358,6 +364,11 @@
         <t>Exactly as on the Roster tab.</t>
       </text>
     </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Minutes played. PLEASE fill this in — it unlocks per-36 stats and minutes load.</t>
+      </text>
+    </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>Field goals made (include 3s)</t>
@@ -406,6 +417,21 @@
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>Personal fouls</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>OPTIONAL: 1 if the player started, else 0.</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>OPTIONAL: deflections.</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>OPTIONAL: charges drawn.</t>
       </text>
     </comment>
   </commentList>
@@ -1559,7 +1585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1579,6 +1605,9 @@
     <col width="6.5" customWidth="1" min="15" max="15"/>
     <col width="6.5" customWidth="1" min="16" max="16"/>
     <col width="6.5" customWidth="1" min="17" max="17"/>
+    <col width="6.5" customWidth="1" min="18" max="18"/>
+    <col width="6.5" customWidth="1" min="19" max="19"/>
+    <col width="6.5" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1667,6 +1696,21 @@
           <t>pf</t>
         </is>
       </c>
+      <c r="R1" s="8" t="inlineStr">
+        <is>
+          <t>started</t>
+        </is>
+      </c>
+      <c r="S1" s="8" t="inlineStr">
+        <is>
+          <t>dfl</t>
+        </is>
+      </c>
+      <c r="T1" s="8" t="inlineStr">
+        <is>
+          <t>chg</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -1680,7 +1724,7 @@
           <t>Christian Towe</t>
         </is>
       </c>
-      <c r="D2" s="15" t="n"/>
+      <c r="D2" s="16" t="n"/>
       <c r="E2" s="15" t="n"/>
       <c r="F2" s="15" t="n"/>
       <c r="G2" s="15" t="n"/>
@@ -1694,6 +1738,9 @@
       <c r="O2" s="15" t="n"/>
       <c r="P2" s="15" t="n"/>
       <c r="Q2" s="15" t="n"/>
+      <c r="R2" s="17" t="n"/>
+      <c r="S2" s="17" t="n"/>
+      <c r="T2" s="17" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -1707,7 +1754,7 @@
           <t>Grant Cage</t>
         </is>
       </c>
-      <c r="D3" s="15" t="n"/>
+      <c r="D3" s="16" t="n"/>
       <c r="E3" s="15" t="n"/>
       <c r="F3" s="15" t="n"/>
       <c r="G3" s="15" t="n"/>
@@ -1721,6 +1768,9 @@
       <c r="O3" s="15" t="n"/>
       <c r="P3" s="15" t="n"/>
       <c r="Q3" s="15" t="n"/>
+      <c r="R3" s="17" t="n"/>
+      <c r="S3" s="17" t="n"/>
+      <c r="T3" s="17" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -1734,7 +1784,7 @@
           <t>Chase Jackson</t>
         </is>
       </c>
-      <c r="D4" s="15" t="n"/>
+      <c r="D4" s="16" t="n"/>
       <c r="E4" s="15" t="n"/>
       <c r="F4" s="15" t="n"/>
       <c r="G4" s="15" t="n"/>
@@ -1748,6 +1798,9 @@
       <c r="O4" s="15" t="n"/>
       <c r="P4" s="15" t="n"/>
       <c r="Q4" s="15" t="n"/>
+      <c r="R4" s="17" t="n"/>
+      <c r="S4" s="17" t="n"/>
+      <c r="T4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -1761,7 +1814,7 @@
           <t>Noah Philips</t>
         </is>
       </c>
-      <c r="D5" s="15" t="n"/>
+      <c r="D5" s="16" t="n"/>
       <c r="E5" s="15" t="n"/>
       <c r="F5" s="15" t="n"/>
       <c r="G5" s="15" t="n"/>
@@ -1775,6 +1828,9 @@
       <c r="O5" s="15" t="n"/>
       <c r="P5" s="15" t="n"/>
       <c r="Q5" s="15" t="n"/>
+      <c r="R5" s="17" t="n"/>
+      <c r="S5" s="17" t="n"/>
+      <c r="T5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1788,7 +1844,7 @@
           <t>Gavin Payne</t>
         </is>
       </c>
-      <c r="D6" s="15" t="n"/>
+      <c r="D6" s="16" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="15" t="n"/>
       <c r="G6" s="15" t="n"/>
@@ -1802,6 +1858,9 @@
       <c r="O6" s="15" t="n"/>
       <c r="P6" s="15" t="n"/>
       <c r="Q6" s="15" t="n"/>
+      <c r="R6" s="17" t="n"/>
+      <c r="S6" s="17" t="n"/>
+      <c r="T6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1815,7 +1874,7 @@
           <t>Elijah Small</t>
         </is>
       </c>
-      <c r="D7" s="15" t="n"/>
+      <c r="D7" s="16" t="n"/>
       <c r="E7" s="15" t="n"/>
       <c r="F7" s="15" t="n"/>
       <c r="G7" s="15" t="n"/>
@@ -1829,6 +1888,9 @@
       <c r="O7" s="15" t="n"/>
       <c r="P7" s="15" t="n"/>
       <c r="Q7" s="15" t="n"/>
+      <c r="R7" s="17" t="n"/>
+      <c r="S7" s="17" t="n"/>
+      <c r="T7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1842,7 +1904,7 @@
           <t>Chris Moore</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n"/>
+      <c r="D8" s="16" t="n"/>
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
@@ -1856,6 +1918,9 @@
       <c r="O8" s="15" t="n"/>
       <c r="P8" s="15" t="n"/>
       <c r="Q8" s="15" t="n"/>
+      <c r="R8" s="17" t="n"/>
+      <c r="S8" s="17" t="n"/>
+      <c r="T8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1869,7 +1934,7 @@
           <t>Leo Thompson</t>
         </is>
       </c>
-      <c r="D9" s="15" t="n"/>
+      <c r="D9" s="16" t="n"/>
       <c r="E9" s="15" t="n"/>
       <c r="F9" s="15" t="n"/>
       <c r="G9" s="15" t="n"/>
@@ -1883,6 +1948,9 @@
       <c r="O9" s="15" t="n"/>
       <c r="P9" s="15" t="n"/>
       <c r="Q9" s="15" t="n"/>
+      <c r="R9" s="17" t="n"/>
+      <c r="S9" s="17" t="n"/>
+      <c r="T9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -1896,7 +1964,7 @@
           <t>Miles Willis</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n"/>
+      <c r="D10" s="16" t="n"/>
       <c r="E10" s="15" t="n"/>
       <c r="F10" s="15" t="n"/>
       <c r="G10" s="15" t="n"/>
@@ -1910,6 +1978,9 @@
       <c r="O10" s="15" t="n"/>
       <c r="P10" s="15" t="n"/>
       <c r="Q10" s="15" t="n"/>
+      <c r="R10" s="17" t="n"/>
+      <c r="S10" s="17" t="n"/>
+      <c r="T10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -1923,7 +1994,7 @@
           <t>Noah Laster</t>
         </is>
       </c>
-      <c r="D11" s="15" t="n"/>
+      <c r="D11" s="16" t="n"/>
       <c r="E11" s="15" t="n"/>
       <c r="F11" s="15" t="n"/>
       <c r="G11" s="15" t="n"/>
@@ -1937,6 +2008,9 @@
       <c r="O11" s="15" t="n"/>
       <c r="P11" s="15" t="n"/>
       <c r="Q11" s="15" t="n"/>
+      <c r="R11" s="17" t="n"/>
+      <c r="S11" s="17" t="n"/>
+      <c r="T11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -1950,7 +2024,7 @@
           <t>Reid Bauman</t>
         </is>
       </c>
-      <c r="D12" s="15" t="n"/>
+      <c r="D12" s="16" t="n"/>
       <c r="E12" s="15" t="n"/>
       <c r="F12" s="15" t="n"/>
       <c r="G12" s="15" t="n"/>
@@ -1964,6 +2038,9 @@
       <c r="O12" s="15" t="n"/>
       <c r="P12" s="15" t="n"/>
       <c r="Q12" s="15" t="n"/>
+      <c r="R12" s="17" t="n"/>
+      <c r="S12" s="17" t="n"/>
+      <c r="T12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1977,7 +2054,7 @@
           <t>Candin Sweet</t>
         </is>
       </c>
-      <c r="D13" s="15" t="n"/>
+      <c r="D13" s="16" t="n"/>
       <c r="E13" s="15" t="n"/>
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="15" t="n"/>
@@ -1991,6 +2068,9 @@
       <c r="O13" s="15" t="n"/>
       <c r="P13" s="15" t="n"/>
       <c r="Q13" s="15" t="n"/>
+      <c r="R13" s="17" t="n"/>
+      <c r="S13" s="17" t="n"/>
+      <c r="T13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -2004,7 +2084,7 @@
           <t>Isaiah Burroughs</t>
         </is>
       </c>
-      <c r="D14" s="15" t="n"/>
+      <c r="D14" s="16" t="n"/>
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n"/>
@@ -2018,6 +2098,9 @@
       <c r="O14" s="15" t="n"/>
       <c r="P14" s="15" t="n"/>
       <c r="Q14" s="15" t="n"/>
+      <c r="R14" s="17" t="n"/>
+      <c r="S14" s="17" t="n"/>
+      <c r="T14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -2031,7 +2114,7 @@
           <t>Sean Colbert</t>
         </is>
       </c>
-      <c r="D15" s="15" t="n"/>
+      <c r="D15" s="16" t="n"/>
       <c r="E15" s="15" t="n"/>
       <c r="F15" s="15" t="n"/>
       <c r="G15" s="15" t="n"/>
@@ -2045,6 +2128,9 @@
       <c r="O15" s="15" t="n"/>
       <c r="P15" s="15" t="n"/>
       <c r="Q15" s="15" t="n"/>
+      <c r="R15" s="17" t="n"/>
+      <c r="S15" s="17" t="n"/>
+      <c r="T15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -2058,7 +2144,7 @@
           <t>Max Sow</t>
         </is>
       </c>
-      <c r="D16" s="15" t="n"/>
+      <c r="D16" s="16" t="n"/>
       <c r="E16" s="15" t="n"/>
       <c r="F16" s="15" t="n"/>
       <c r="G16" s="15" t="n"/>
@@ -2072,6 +2158,9 @@
       <c r="O16" s="15" t="n"/>
       <c r="P16" s="15" t="n"/>
       <c r="Q16" s="15" t="n"/>
+      <c r="R16" s="17" t="n"/>
+      <c r="S16" s="17" t="n"/>
+      <c r="T16" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">

</xml_diff>